<commit_message>
add commitment proof employer to contract
</commit_message>
<xml_diff>
--- a/roster-template.xlsx
+++ b/roster-template.xlsx
@@ -11,7 +11,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>Payroll period</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
   <si>
     <t>Full name</t>
   </si>
@@ -28,88 +37,58 @@
     <t>Keizersgracht 12, 1015 CW Amsterdam</t>
   </si>
   <si>
-    <t>4200.00</t>
-  </si>
-  <si>
     <t>Bram Jansen</t>
   </si>
   <si>
     <t>Lange Voorhout 3, 2514 EA Den Haag</t>
   </si>
   <si>
-    <t>3850.50</t>
-  </si>
-  <si>
     <t>Chiara Rossi</t>
   </si>
   <si>
     <t>Via Roma 44, 20121 Milano</t>
   </si>
   <si>
-    <t>5100.00</t>
-  </si>
-  <si>
     <t>Daan Bakker</t>
   </si>
   <si>
     <t>Coolsingel 210, 3012 AG Rotterdam</t>
   </si>
   <si>
-    <t>3600.00</t>
-  </si>
-  <si>
     <t>Elif Yilmaz</t>
   </si>
   <si>
     <t>Bahariye Cd. 8, 34710 Istanbul</t>
   </si>
   <si>
-    <t>4475.25</t>
-  </si>
-  <si>
     <t>Femke Visser</t>
   </si>
   <si>
     <t>Oudegracht 91, 3511 AE Utrecht</t>
   </si>
   <si>
-    <t>3990.00</t>
-  </si>
-  <si>
     <t>Gideon Okafor</t>
   </si>
   <si>
     <t>Adeola Odeku St 17, Lagos</t>
   </si>
   <si>
-    <t>4720.00</t>
-  </si>
-  <si>
     <t>Hanna Nowak</t>
   </si>
   <si>
     <t>Ulica Floriańska 5, 31-019 Kraków</t>
   </si>
   <si>
-    <t>3410.75</t>
-  </si>
-  <si>
     <t>Ivo Novák</t>
   </si>
   <si>
     <t>Národní 22, 110 00 Praha</t>
   </si>
   <si>
-    <t>3125.00</t>
-  </si>
-  <si>
     <t>Julia Meijer</t>
   </si>
   <si>
     <t>Grote Markt 7, 9711 LV Groningen</t>
-  </si>
-  <si>
-    <t>5300.00</t>
   </si>
 </sst>
 </file>
@@ -148,10 +127,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -492,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -500,128 +480,157 @@
     <col min="3" max="3" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4200</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3850.5</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5100</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3600</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
+      </c>
+      <c r="C9" s="1">
+        <v>4475.25</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
+      </c>
+      <c r="C10" s="1">
+        <v>3990</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>19</v>
+      </c>
+      <c r="C11" s="1">
+        <v>4720</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3410.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="1">
+        <v>3125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1">
+        <v>5300</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="whole" showErrorMessage="1" errorTitle="Year" error="Use a four-digit year, e.g. 2026." sqref="C1">
+      <formula1>2000</formula1>
+      <formula2>2999</formula2>
+    </dataValidation>
+    <dataValidation type="whole" showErrorMessage="1" errorTitle="Month" error="Use a month number from 1 to 12." sqref="C2">
+      <formula1>1</formula1>
+      <formula2>12</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Sending pEUR in the smartcontract privately via browser!
</commit_message>
<xml_diff>
--- a/roster-template.xlsx
+++ b/roster-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Payroll period</t>
   </si>
@@ -41,54 +41,6 @@
   </si>
   <si>
     <t>Lange Voorhout 3, 2514 EA Den Haag</t>
-  </si>
-  <si>
-    <t>Chiara Rossi</t>
-  </si>
-  <si>
-    <t>Via Roma 44, 20121 Milano</t>
-  </si>
-  <si>
-    <t>Daan Bakker</t>
-  </si>
-  <si>
-    <t>Coolsingel 210, 3012 AG Rotterdam</t>
-  </si>
-  <si>
-    <t>Elif Yilmaz</t>
-  </si>
-  <si>
-    <t>Bahariye Cd. 8, 34710 Istanbul</t>
-  </si>
-  <si>
-    <t>Femke Visser</t>
-  </si>
-  <si>
-    <t>Oudegracht 91, 3511 AE Utrecht</t>
-  </si>
-  <si>
-    <t>Gideon Okafor</t>
-  </si>
-  <si>
-    <t>Adeola Odeku St 17, Lagos</t>
-  </si>
-  <si>
-    <t>Hanna Nowak</t>
-  </si>
-  <si>
-    <t>Ulica Floriańska 5, 31-019 Kraków</t>
-  </si>
-  <si>
-    <t>Ivo Novák</t>
-  </si>
-  <si>
-    <t>Národní 22, 110 00 Praha</t>
-  </si>
-  <si>
-    <t>Julia Meijer</t>
-  </si>
-  <si>
-    <t>Grote Markt 7, 9711 LV Groningen</t>
   </si>
 </sst>
 </file>
@@ -472,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -530,94 +482,6 @@
       </c>
       <c r="C6" s="1">
         <v>3850.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="1">
-        <v>5100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="1">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="1">
-        <v>4475.25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="1">
-        <v>3990</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="1">
-        <v>4720</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1">
-        <v>3410.75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="1">
-        <v>3125</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="1">
-        <v>5300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>